<commit_message>
20251223: New DRC for Drawing Layers
</commit_message>
<xml_diff>
--- a/Document/Layer_Tables/TR-1um_GDSII_Table.xlsx
+++ b/Document/Layer_Tables/TR-1um_GDSII_Table.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/Layer_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{876F3FE8-95CD-1E4F-A1C5-E7741EC17A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9FA724-DF0D-9A4C-BC42-16F040CBEDFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="1060" windowWidth="33120" windowHeight="27580" activeTab="1" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="840" yWindow="760" windowWidth="29400" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
-    <sheet name="DR (Drawing)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="103">
   <si>
     <t>PSUB</t>
   </si>
@@ -346,511 +345,13 @@
   </si>
   <si>
     <t>PO</t>
-  </si>
-  <si>
-    <t>WN.W1</t>
-  </si>
-  <si>
-    <t>WN.S1</t>
-  </si>
-  <si>
-    <t>WN.S2</t>
-  </si>
-  <si>
-    <t>WN.S3</t>
-  </si>
-  <si>
-    <t>WN.S4</t>
-  </si>
-  <si>
-    <t>WN.S5</t>
-  </si>
-  <si>
-    <t>WN.S6</t>
-  </si>
-  <si>
-    <t>WN.AP</t>
-  </si>
-  <si>
-    <t>WN.AN</t>
-  </si>
-  <si>
-    <t>ER0001</t>
-  </si>
-  <si>
-    <t>ER0104</t>
-  </si>
-  <si>
-    <t>WN-WN Smin</t>
-  </si>
-  <si>
-    <t>WN-AN Smin</t>
-  </si>
-  <si>
-    <t>ER0132</t>
-  </si>
-  <si>
-    <t>ER0128</t>
-  </si>
-  <si>
-    <t>ER0130</t>
-  </si>
-  <si>
-    <t>ER0129</t>
-  </si>
-  <si>
-    <t>ER0122</t>
-  </si>
-  <si>
-    <t>WN-AP Smin</t>
-  </si>
-  <si>
-    <t>AP.WN</t>
-  </si>
-  <si>
-    <t>AN.WN</t>
-  </si>
-  <si>
-    <t>AP-WN Emin</t>
-  </si>
-  <si>
-    <t>AN-WN Emin</t>
-  </si>
-  <si>
-    <t>ERWLMN01</t>
-  </si>
-  <si>
-    <t>ERWLMN03</t>
-  </si>
-  <si>
-    <t>AR.W1</t>
-  </si>
-  <si>
-    <t>AR.S1</t>
-  </si>
-  <si>
-    <t>AR.WR</t>
-  </si>
-  <si>
-    <t>AN.WR</t>
-  </si>
-  <si>
-    <t>AR.AN</t>
-  </si>
-  <si>
-    <t>ERWLMP02</t>
-  </si>
-  <si>
-    <t>ERWLMP03</t>
-  </si>
-  <si>
-    <t>AR Wmin</t>
-  </si>
-  <si>
-    <t>WN Wmin</t>
-  </si>
-  <si>
-    <t>AR Smin</t>
-  </si>
-  <si>
-    <t>AR-WN(R) Emin</t>
-  </si>
-  <si>
-    <t>AR-AN Smin</t>
-  </si>
-  <si>
-    <t>ERRR07</t>
-  </si>
-  <si>
-    <t>ERWLRR02</t>
-  </si>
-  <si>
-    <t>ERWLRR03</t>
-  </si>
-  <si>
-    <t>AN-WN(R) Emin</t>
-  </si>
-  <si>
-    <t>ERWLRR01</t>
-  </si>
-  <si>
-    <t>ERWLRR04</t>
-  </si>
-  <si>
-    <t>AC.W1</t>
-  </si>
-  <si>
-    <t>AC.S1</t>
-  </si>
-  <si>
-    <t>AC.WC</t>
-  </si>
-  <si>
-    <t>AN.WC</t>
-  </si>
-  <si>
-    <t>AC.AN</t>
-  </si>
-  <si>
-    <t>AC-AN Smin</t>
-  </si>
-  <si>
-    <t>AC-WN(C) Emin</t>
-  </si>
-  <si>
-    <t>WN-WN(R) Smin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WN-WN(C) Smin </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WN(R)-WN(C) Smin </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WN(R)-WN(R) Smin </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WN(C)-WN(C) Smin </t>
-  </si>
-  <si>
-    <t>AC Wmin</t>
-  </si>
-  <si>
-    <t>AC Smin</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>AN-WN(C) Emin</t>
-  </si>
-  <si>
-    <t>ERCSIO04</t>
-  </si>
-  <si>
-    <t>ERCSIO11</t>
-  </si>
-  <si>
-    <t>AP.W1</t>
-  </si>
-  <si>
-    <t>AP.S1</t>
-  </si>
-  <si>
-    <t>AP.AN</t>
-  </si>
-  <si>
-    <t>AP.WM</t>
-  </si>
-  <si>
-    <t>AP Wmin</t>
-  </si>
-  <si>
-    <t>AP Smin</t>
-  </si>
-  <si>
-    <t>AP-AN Smin</t>
-  </si>
-  <si>
-    <t>PMOS Wmin</t>
-  </si>
-  <si>
-    <t>AN.W1</t>
-  </si>
-  <si>
-    <t>AN.S1</t>
-  </si>
-  <si>
-    <t>AN.WM</t>
-  </si>
-  <si>
-    <t>NMOS Wmin</t>
-  </si>
-  <si>
-    <t>AN Wmin</t>
-  </si>
-  <si>
-    <t>AN Smin</t>
-  </si>
-  <si>
-    <t>AN.AP</t>
-  </si>
-  <si>
-    <t>AN-AP Smin</t>
-  </si>
-  <si>
-    <t>DP.W1</t>
-  </si>
-  <si>
-    <t>DP.S1</t>
-  </si>
-  <si>
-    <t>DP.AP</t>
-  </si>
-  <si>
-    <t>DP.AN</t>
-  </si>
-  <si>
-    <t>DP-AP Smin</t>
-  </si>
-  <si>
-    <t>DP-AN Smin</t>
-  </si>
-  <si>
-    <t>DN.S1</t>
-  </si>
-  <si>
-    <t>DN.AP</t>
-  </si>
-  <si>
-    <t>DN.AN</t>
-  </si>
-  <si>
-    <t>DN Smin</t>
-  </si>
-  <si>
-    <t>ERWLMP08</t>
-  </si>
-  <si>
-    <t>ERWLMP09</t>
-  </si>
-  <si>
-    <t>ER0028</t>
-  </si>
-  <si>
-    <t>ER0004</t>
-  </si>
-  <si>
-    <t>ERWLMP04</t>
-  </si>
-  <si>
-    <t>ERMP13</t>
-  </si>
-  <si>
-    <t>???</t>
-  </si>
-  <si>
-    <t>ERWLMN05</t>
-  </si>
-  <si>
-    <t>ERMN15</t>
-  </si>
-  <si>
-    <t>ERWLMN10</t>
-  </si>
-  <si>
-    <t>ERWLMN11</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>PO.W1</t>
-  </si>
-  <si>
-    <t>PO.S1</t>
-  </si>
-  <si>
-    <t>PO.AP</t>
-  </si>
-  <si>
-    <t>PO.AN</t>
-  </si>
-  <si>
-    <t>PO.EM</t>
-  </si>
-  <si>
-    <t>PO Wmin</t>
-  </si>
-  <si>
-    <t>PO Smin</t>
-  </si>
-  <si>
-    <t>PO-AP Smin</t>
-  </si>
-  <si>
-    <t>PO-AN Smin</t>
-  </si>
-  <si>
-    <t>CO.W1</t>
-  </si>
-  <si>
-    <t>CO.S1</t>
-  </si>
-  <si>
-    <t>CO.WD</t>
-  </si>
-  <si>
-    <t>CO(D) Width</t>
-  </si>
-  <si>
-    <t>CO Wmin</t>
-  </si>
-  <si>
-    <t>CO Smin</t>
-  </si>
-  <si>
-    <t>CO.AN</t>
-  </si>
-  <si>
-    <t>CO.AP</t>
-  </si>
-  <si>
-    <t>CO-AP Emin</t>
-  </si>
-  <si>
-    <t>CO-AN Emin</t>
-  </si>
-  <si>
-    <t>CO.PG</t>
-  </si>
-  <si>
-    <t>CO.PO</t>
-  </si>
-  <si>
-    <t>CO-PO(G) Smin</t>
-  </si>
-  <si>
-    <t>CO-PO Emin</t>
-  </si>
-  <si>
-    <t>CO.AD</t>
-  </si>
-  <si>
-    <t>CO-AD Emin</t>
-  </si>
-  <si>
-    <t>CC.W1</t>
-  </si>
-  <si>
-    <t>CC.S1</t>
-  </si>
-  <si>
-    <t>CC.AC</t>
-  </si>
-  <si>
-    <t>CC.AN</t>
-  </si>
-  <si>
-    <t>CO(C) Wmin</t>
-  </si>
-  <si>
-    <t>CO(C) Smin</t>
-  </si>
-  <si>
-    <t>CO(C)-AC Emin</t>
-  </si>
-  <si>
-    <t>CO(C)-AN Emim</t>
-  </si>
-  <si>
-    <t>M1.W1</t>
-  </si>
-  <si>
-    <t>M1.S1</t>
-  </si>
-  <si>
-    <t>M1.S2</t>
-  </si>
-  <si>
-    <t>M1 Wmin</t>
-  </si>
-  <si>
-    <t>M1 Smin</t>
-  </si>
-  <si>
-    <t>M1(W) Wmin</t>
-  </si>
-  <si>
-    <t>M1(W) Smin</t>
-  </si>
-  <si>
-    <t>M1.CO</t>
-  </si>
-  <si>
-    <t>M1.CC</t>
-  </si>
-  <si>
-    <t>V1.W1</t>
-  </si>
-  <si>
-    <t>V1.S1</t>
-  </si>
-  <si>
-    <t>V1.M1</t>
-  </si>
-  <si>
-    <t>V1.PO</t>
-  </si>
-  <si>
-    <t>V1.CO</t>
-  </si>
-  <si>
-    <t>V1.CL</t>
-  </si>
-  <si>
-    <t>M2.W1</t>
-  </si>
-  <si>
-    <t>M2.W2</t>
-  </si>
-  <si>
-    <t>M2.V1</t>
-  </si>
-  <si>
-    <t>V1 Windth</t>
-  </si>
-  <si>
-    <t>V1 Smin</t>
-  </si>
-  <si>
-    <t>V1-M1 Emin</t>
-  </si>
-  <si>
-    <t>V1-PO Smin</t>
-  </si>
-  <si>
-    <t>V1-CO Smin</t>
-  </si>
-  <si>
-    <t>V1-CO(L) Smin</t>
-  </si>
-  <si>
-    <t>M2 Wmin</t>
-  </si>
-  <si>
-    <t>M2 Smin</t>
-  </si>
-  <si>
-    <t>M1-CO Omin</t>
-  </si>
-  <si>
-    <t>M1-CO(C) Omin</t>
-  </si>
-  <si>
-    <t>M2-V1 Omin</t>
-  </si>
-  <si>
-    <t>Rule</t>
-  </si>
-  <si>
-    <t>IP62 Rule Name</t>
-  </si>
-  <si>
-    <t>DP Smin</t>
-  </si>
-  <si>
-    <t>MOS Endcap min</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -885,32 +386,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Courier New"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Courier New"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Courier New"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="9"/>
-      <name val="Courier New"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -951,7 +426,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -1207,26 +682,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1414,24 +874,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1458,39 +900,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1507,389 +916,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>10949</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>208018</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>87586</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E77C5B0E-0284-F194-9C18-41A3A8EA0C1E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7488621" y="208018"/>
-          <a:ext cx="3361120" cy="2189654"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="accent5">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Note:</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:br>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Wmin:	Width min</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Smin</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> :	</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Space min</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Emin:	Enclosure min</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Omin</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>:	</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Fringe min</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Windth:	Windth equal</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t>Space:	Space equal</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1600">
-              <a:effectLst/>
-              <a:latin typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-              <a:cs typeface="Courier New" panose="02070309020205020404" pitchFamily="49" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1600"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2225,17 +1251,17 @@
     <row r="1" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:13" s="3" customFormat="1" ht="22" x14ac:dyDescent="0.2">
       <c r="B2" s="28"/>
-      <c r="C2" s="69" t="s">
+      <c r="C2" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="70"/>
-      <c r="E2" s="71"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="65"/>
       <c r="F2" s="29"/>
-      <c r="G2" s="72" t="s">
+      <c r="G2" s="66" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="73"/>
-      <c r="I2" s="74"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="68"/>
       <c r="J2" s="29"/>
       <c r="K2" s="29"/>
       <c r="L2" s="29"/>
@@ -3159,11 +2185,11 @@
     </row>
     <row r="43" spans="2:13" ht="22" x14ac:dyDescent="0.2">
       <c r="B43" s="23"/>
-      <c r="C43" s="75" t="s">
+      <c r="C43" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="77"/>
+      <c r="D43" s="70"/>
+      <c r="E43" s="71"/>
       <c r="F43" s="24"/>
       <c r="G43" s="25"/>
       <c r="H43" s="24"/>
@@ -3664,949 +2690,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:E77"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="4.6640625" style="63" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="63"/>
-    <col min="3" max="3" width="32.33203125" style="64" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="65"/>
-    <col min="5" max="5" width="28.83203125" style="63" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="63"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="78" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="79" t="s">
-        <v>201</v>
-      </c>
-      <c r="D2" s="80" t="s">
-        <v>264</v>
-      </c>
-      <c r="E2" s="78" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B3" s="81" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="82" t="s">
-        <v>136</v>
-      </c>
-      <c r="D3" s="83">
-        <v>8</v>
-      </c>
-      <c r="E3" s="81" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B4" s="81" t="s">
-        <v>104</v>
-      </c>
-      <c r="C4" s="84" t="s">
-        <v>114</v>
-      </c>
-      <c r="D4" s="83">
-        <v>12</v>
-      </c>
-      <c r="E4" s="81" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B5" s="81" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" s="84" t="s">
-        <v>153</v>
-      </c>
-      <c r="D5" s="83">
-        <v>9.5</v>
-      </c>
-      <c r="E5" s="85" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B6" s="81" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="84" t="s">
-        <v>154</v>
-      </c>
-      <c r="D6" s="83">
-        <v>12</v>
-      </c>
-      <c r="E6" s="85" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B7" s="81" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" s="84" t="s">
-        <v>155</v>
-      </c>
-      <c r="D7" s="83">
-        <v>9.5</v>
-      </c>
-      <c r="E7" s="85" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B8" s="81" t="s">
-        <v>108</v>
-      </c>
-      <c r="C8" s="84" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="83">
-        <v>8</v>
-      </c>
-      <c r="E8" s="85" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B9" s="81" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" s="84" t="s">
-        <v>157</v>
-      </c>
-      <c r="D9" s="83">
-        <v>12</v>
-      </c>
-      <c r="E9" s="85" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B10" s="81" t="s">
-        <v>110</v>
-      </c>
-      <c r="C10" s="84" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10" s="83">
-        <v>10</v>
-      </c>
-      <c r="E10" s="85" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B11" s="81" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="84" t="s">
-        <v>115</v>
-      </c>
-      <c r="D11" s="83">
-        <v>5</v>
-      </c>
-      <c r="E11" s="85" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B12" s="86" t="s">
-        <v>164</v>
-      </c>
-      <c r="C12" s="87" t="s">
-        <v>168</v>
-      </c>
-      <c r="D12" s="88">
-        <v>1.4</v>
-      </c>
-      <c r="E12" s="86" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B13" s="86" t="s">
-        <v>165</v>
-      </c>
-      <c r="C13" s="87" t="s">
-        <v>169</v>
-      </c>
-      <c r="D13" s="88">
-        <v>1.4</v>
-      </c>
-      <c r="E13" s="86" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B14" s="86" t="s">
-        <v>166</v>
-      </c>
-      <c r="C14" s="87" t="s">
-        <v>170</v>
-      </c>
-      <c r="D14" s="88">
-        <v>2.8</v>
-      </c>
-      <c r="E14" s="86" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B15" s="86" t="s">
-        <v>167</v>
-      </c>
-      <c r="C15" s="87" t="s">
-        <v>171</v>
-      </c>
-      <c r="D15" s="88">
-        <v>3.4</v>
-      </c>
-      <c r="E15" s="86" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B16" s="86" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" s="87" t="s">
-        <v>124</v>
-      </c>
-      <c r="D16" s="88">
-        <v>7</v>
-      </c>
-      <c r="E16" s="86" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="86" t="s">
-        <v>180</v>
-      </c>
-      <c r="C17" s="87" t="s">
-        <v>168</v>
-      </c>
-      <c r="D17" s="88">
-        <v>1.4</v>
-      </c>
-      <c r="E17" s="86" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18" s="86" t="s">
-        <v>181</v>
-      </c>
-      <c r="C18" s="87" t="s">
-        <v>266</v>
-      </c>
-      <c r="D18" s="88" t="s">
-        <v>160</v>
-      </c>
-      <c r="E18" s="86" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19" s="86" t="s">
-        <v>182</v>
-      </c>
-      <c r="C19" s="87" t="s">
-        <v>184</v>
-      </c>
-      <c r="D19" s="88">
-        <v>2.8</v>
-      </c>
-      <c r="E19" s="86" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="86" t="s">
-        <v>183</v>
-      </c>
-      <c r="C20" s="87" t="s">
-        <v>185</v>
-      </c>
-      <c r="D20" s="88">
-        <v>2.8</v>
-      </c>
-      <c r="E20" s="86" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21" s="81" t="s">
-        <v>172</v>
-      </c>
-      <c r="C21" s="82" t="s">
-        <v>176</v>
-      </c>
-      <c r="D21" s="83">
-        <v>1.4</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B22" s="81" t="s">
-        <v>173</v>
-      </c>
-      <c r="C22" s="82" t="s">
-        <v>177</v>
-      </c>
-      <c r="D22" s="83">
-        <v>1.4</v>
-      </c>
-      <c r="E22" s="81" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" s="81" t="s">
-        <v>178</v>
-      </c>
-      <c r="C23" s="82" t="s">
-        <v>179</v>
-      </c>
-      <c r="D23" s="83">
-        <v>2.8</v>
-      </c>
-      <c r="E23" s="81" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" s="81" t="s">
-        <v>174</v>
-      </c>
-      <c r="C24" s="82" t="s">
-        <v>175</v>
-      </c>
-      <c r="D24" s="83">
-        <v>3.4</v>
-      </c>
-      <c r="E24" s="81" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" s="81" t="s">
-        <v>123</v>
-      </c>
-      <c r="C25" s="82" t="s">
-        <v>125</v>
-      </c>
-      <c r="D25" s="83">
-        <v>5</v>
-      </c>
-      <c r="E25" s="81" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B26" s="81" t="s">
-        <v>186</v>
-      </c>
-      <c r="C26" s="82" t="s">
-        <v>189</v>
-      </c>
-      <c r="D26" s="83" t="s">
-        <v>160</v>
-      </c>
-      <c r="E26" s="81" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B27" s="81" t="s">
-        <v>187</v>
-      </c>
-      <c r="C27" s="82" t="s">
-        <v>184</v>
-      </c>
-      <c r="D27" s="83">
-        <v>2.8</v>
-      </c>
-      <c r="E27" s="81" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="28" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="81" t="s">
-        <v>188</v>
-      </c>
-      <c r="C28" s="82" t="s">
-        <v>185</v>
-      </c>
-      <c r="D28" s="83">
-        <v>2.8</v>
-      </c>
-      <c r="E28" s="81" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B29" s="86" t="s">
-        <v>128</v>
-      </c>
-      <c r="C29" s="87" t="s">
-        <v>135</v>
-      </c>
-      <c r="D29" s="88">
-        <v>2.8</v>
-      </c>
-      <c r="E29" s="86" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B30" s="86" t="s">
-        <v>129</v>
-      </c>
-      <c r="C30" s="87" t="s">
-        <v>137</v>
-      </c>
-      <c r="D30" s="88">
-        <v>4</v>
-      </c>
-      <c r="E30" s="86" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B31" s="86" t="s">
-        <v>130</v>
-      </c>
-      <c r="C31" s="87" t="s">
-        <v>138</v>
-      </c>
-      <c r="D31" s="88">
-        <v>10</v>
-      </c>
-      <c r="E31" s="86" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B32" s="86" t="s">
-        <v>131</v>
-      </c>
-      <c r="C32" s="87" t="s">
-        <v>143</v>
-      </c>
-      <c r="D32" s="88">
-        <v>10</v>
-      </c>
-      <c r="E32" s="86" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B33" s="81" t="s">
-        <v>132</v>
-      </c>
-      <c r="C33" s="82" t="s">
-        <v>139</v>
-      </c>
-      <c r="D33" s="83">
-        <v>4</v>
-      </c>
-      <c r="E33" s="81" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="81" t="s">
-        <v>146</v>
-      </c>
-      <c r="C34" s="82" t="s">
-        <v>158</v>
-      </c>
-      <c r="D34" s="83" t="s">
-        <v>160</v>
-      </c>
-      <c r="E34" s="81"/>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="81" t="s">
-        <v>147</v>
-      </c>
-      <c r="C35" s="82" t="s">
-        <v>159</v>
-      </c>
-      <c r="D35" s="83" t="s">
-        <v>160</v>
-      </c>
-      <c r="E35" s="81"/>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B36" s="81" t="s">
-        <v>148</v>
-      </c>
-      <c r="C36" s="82" t="s">
-        <v>152</v>
-      </c>
-      <c r="D36" s="83" t="s">
-        <v>160</v>
-      </c>
-      <c r="E36" s="81"/>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B37" s="81" t="s">
-        <v>149</v>
-      </c>
-      <c r="C37" s="82" t="s">
-        <v>161</v>
-      </c>
-      <c r="D37" s="83">
-        <v>3</v>
-      </c>
-      <c r="E37" s="81" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B38" s="81" t="s">
-        <v>150</v>
-      </c>
-      <c r="C38" s="82" t="s">
-        <v>151</v>
-      </c>
-      <c r="D38" s="83">
-        <v>2.8</v>
-      </c>
-      <c r="E38" s="81" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B39" s="86" t="s">
-        <v>202</v>
-      </c>
-      <c r="C39" s="87" t="s">
-        <v>207</v>
-      </c>
-      <c r="D39" s="88">
-        <v>1</v>
-      </c>
-      <c r="E39" s="86"/>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B40" s="86" t="s">
-        <v>203</v>
-      </c>
-      <c r="C40" s="87" t="s">
-        <v>208</v>
-      </c>
-      <c r="D40" s="88">
-        <v>1.2</v>
-      </c>
-      <c r="E40" s="86"/>
-    </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B41" s="86" t="s">
-        <v>204</v>
-      </c>
-      <c r="C41" s="87" t="s">
-        <v>209</v>
-      </c>
-      <c r="D41" s="88">
-        <v>0.4</v>
-      </c>
-      <c r="E41" s="86"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B42" s="86" t="s">
-        <v>205</v>
-      </c>
-      <c r="C42" s="87" t="s">
-        <v>210</v>
-      </c>
-      <c r="D42" s="88">
-        <v>0.4</v>
-      </c>
-      <c r="E42" s="86"/>
-    </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B43" s="86" t="s">
-        <v>206</v>
-      </c>
-      <c r="C43" s="87" t="s">
-        <v>267</v>
-      </c>
-      <c r="D43" s="88">
-        <v>1.2</v>
-      </c>
-      <c r="E43" s="86"/>
-    </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B44" s="81" t="s">
-        <v>211</v>
-      </c>
-      <c r="C44" s="82" t="s">
-        <v>215</v>
-      </c>
-      <c r="D44" s="83">
-        <v>1</v>
-      </c>
-      <c r="E44" s="81"/>
-    </row>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B45" s="81" t="s">
-        <v>212</v>
-      </c>
-      <c r="C45" s="82" t="s">
-        <v>216</v>
-      </c>
-      <c r="D45" s="83">
-        <v>1</v>
-      </c>
-      <c r="E45" s="81"/>
-    </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B46" s="81" t="s">
-        <v>213</v>
-      </c>
-      <c r="C46" s="82" t="s">
-        <v>214</v>
-      </c>
-      <c r="D46" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E46" s="81"/>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B47" s="81" t="s">
-        <v>218</v>
-      </c>
-      <c r="C47" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="D47" s="83">
-        <v>0.8</v>
-      </c>
-      <c r="E47" s="81"/>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B48" s="81" t="s">
-        <v>217</v>
-      </c>
-      <c r="C48" s="82" t="s">
-        <v>220</v>
-      </c>
-      <c r="D48" s="83">
-        <v>0.8</v>
-      </c>
-      <c r="E48" s="81"/>
-    </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B49" s="81" t="s">
-        <v>221</v>
-      </c>
-      <c r="C49" s="82" t="s">
-        <v>223</v>
-      </c>
-      <c r="D49" s="83">
-        <v>1</v>
-      </c>
-      <c r="E49" s="81"/>
-    </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B50" s="81" t="s">
-        <v>222</v>
-      </c>
-      <c r="C50" s="82" t="s">
-        <v>224</v>
-      </c>
-      <c r="D50" s="83">
-        <v>0.8</v>
-      </c>
-      <c r="E50" s="81"/>
-    </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B51" s="81" t="s">
-        <v>225</v>
-      </c>
-      <c r="C51" s="82" t="s">
-        <v>226</v>
-      </c>
-      <c r="D51" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E51" s="81"/>
-    </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B52" s="81" t="s">
-        <v>227</v>
-      </c>
-      <c r="C52" s="82" t="s">
-        <v>231</v>
-      </c>
-      <c r="D52" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E52" s="81"/>
-    </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B53" s="81" t="s">
-        <v>228</v>
-      </c>
-      <c r="C53" s="82" t="s">
-        <v>232</v>
-      </c>
-      <c r="D53" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E53" s="81"/>
-    </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B54" s="81" t="s">
-        <v>229</v>
-      </c>
-      <c r="C54" s="82" t="s">
-        <v>233</v>
-      </c>
-      <c r="D54" s="83">
-        <v>2.9</v>
-      </c>
-      <c r="E54" s="81"/>
-    </row>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B55" s="81" t="s">
-        <v>230</v>
-      </c>
-      <c r="C55" s="82" t="s">
-        <v>234</v>
-      </c>
-      <c r="D55" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E55" s="81"/>
-    </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="86" t="s">
-        <v>235</v>
-      </c>
-      <c r="C56" s="87" t="s">
-        <v>238</v>
-      </c>
-      <c r="D56" s="88">
-        <v>1.8</v>
-      </c>
-      <c r="E56" s="86"/>
-    </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B57" s="86" t="s">
-        <v>236</v>
-      </c>
-      <c r="C57" s="87" t="s">
-        <v>239</v>
-      </c>
-      <c r="D57" s="88">
-        <v>1.4</v>
-      </c>
-      <c r="E57" s="86"/>
-    </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B58" s="86" t="s">
-        <v>235</v>
-      </c>
-      <c r="C58" s="87" t="s">
-        <v>240</v>
-      </c>
-      <c r="D58" s="88">
-        <v>10</v>
-      </c>
-      <c r="E58" s="86"/>
-    </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B59" s="86" t="s">
-        <v>237</v>
-      </c>
-      <c r="C59" s="87" t="s">
-        <v>241</v>
-      </c>
-      <c r="D59" s="88">
-        <v>2</v>
-      </c>
-      <c r="E59" s="86"/>
-    </row>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B60" s="86" t="s">
-        <v>242</v>
-      </c>
-      <c r="C60" s="87" t="s">
-        <v>261</v>
-      </c>
-      <c r="D60" s="88">
-        <v>1</v>
-      </c>
-      <c r="E60" s="86"/>
-    </row>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B61" s="86" t="s">
-        <v>243</v>
-      </c>
-      <c r="C61" s="87" t="s">
-        <v>262</v>
-      </c>
-      <c r="D61" s="88">
-        <v>1.2</v>
-      </c>
-      <c r="E61" s="86"/>
-    </row>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B62" s="81" t="s">
-        <v>244</v>
-      </c>
-      <c r="C62" s="82" t="s">
-        <v>253</v>
-      </c>
-      <c r="D62" s="83">
-        <v>1.4</v>
-      </c>
-      <c r="E62" s="81"/>
-    </row>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B63" s="81" t="s">
-        <v>245</v>
-      </c>
-      <c r="C63" s="82" t="s">
-        <v>254</v>
-      </c>
-      <c r="D63" s="83">
-        <v>1.5</v>
-      </c>
-      <c r="E63" s="81"/>
-    </row>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B64" s="81" t="s">
-        <v>246</v>
-      </c>
-      <c r="C64" s="82" t="s">
-        <v>255</v>
-      </c>
-      <c r="D64" s="83">
-        <v>1</v>
-      </c>
-      <c r="E64" s="81"/>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="81" t="s">
-        <v>247</v>
-      </c>
-      <c r="C65" s="82" t="s">
-        <v>256</v>
-      </c>
-      <c r="D65" s="83">
-        <v>1.2</v>
-      </c>
-      <c r="E65" s="81"/>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B66" s="81" t="s">
-        <v>248</v>
-      </c>
-      <c r="C66" s="82" t="s">
-        <v>257</v>
-      </c>
-      <c r="D66" s="83">
-        <v>1</v>
-      </c>
-      <c r="E66" s="81"/>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B67" s="81" t="s">
-        <v>249</v>
-      </c>
-      <c r="C67" s="82" t="s">
-        <v>258</v>
-      </c>
-      <c r="D67" s="83">
-        <v>1.4</v>
-      </c>
-      <c r="E67" s="81"/>
-    </row>
-    <row r="68" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B68" s="86" t="s">
-        <v>250</v>
-      </c>
-      <c r="C68" s="87" t="s">
-        <v>259</v>
-      </c>
-      <c r="D68" s="88">
-        <v>3</v>
-      </c>
-      <c r="E68" s="86"/>
-    </row>
-    <row r="69" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B69" s="86" t="s">
-        <v>251</v>
-      </c>
-      <c r="C69" s="87" t="s">
-        <v>260</v>
-      </c>
-      <c r="D69" s="88">
-        <v>2</v>
-      </c>
-      <c r="E69" s="86"/>
-    </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B70" s="86" t="s">
-        <v>252</v>
-      </c>
-      <c r="C70" s="87" t="s">
-        <v>263</v>
-      </c>
-      <c r="D70" s="88">
-        <v>1</v>
-      </c>
-      <c r="E70" s="86"/>
-    </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B72" s="66"/>
-      <c r="C72" s="68"/>
-      <c r="D72" s="67"/>
-    </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B73" s="66"/>
-      <c r="C73" s="68"/>
-      <c r="D73" s="67"/>
-    </row>
-    <row r="74" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B74" s="66"/>
-      <c r="C74" s="68"/>
-      <c r="D74" s="67"/>
-    </row>
-    <row r="75" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B75" s="66"/>
-      <c r="C75" s="68"/>
-      <c r="D75" s="67"/>
-    </row>
-    <row r="76" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B76" s="66"/>
-      <c r="C76" s="68"/>
-      <c r="D76" s="67"/>
-    </row>
-    <row r="77" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B77" s="66"/>
-      <c r="C77" s="68"/>
-      <c r="D77" s="67"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>